<commit_message>
Completed general medal count for nations, added logs for MLB/NBA clubs
</commit_message>
<xml_diff>
--- a/Example_medals.xlsx
+++ b/Example_medals.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Olympics Simulator v3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\Olympics Simulator v3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA6C2D50-7FD3-41AF-95B0-198861BD09CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EA2BE18-D57C-4DCB-8D54-81CD3712B5A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="6">
   <si>
     <t>Prueba 1</t>
   </si>
@@ -84,8 +84,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -104,12 +107,24 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{38EA0D5D-03F6-4825-ADDF-9ABF3352EDE4}" name="Tabla1" displayName="Tabla1" ref="A1:C4" totalsRowShown="0">
-  <autoFilter ref="A1:C4" xr:uid="{38EA0D5D-03F6-4825-ADDF-9ABF3352EDE4}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{38EA0D5D-03F6-4825-ADDF-9ABF3352EDE4}" name="Tabla1" displayName="Tabla1" ref="A2:C5" totalsRowShown="0">
+  <autoFilter ref="A2:C5" xr:uid="{38EA0D5D-03F6-4825-ADDF-9ABF3352EDE4}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{92133F89-C3BE-4B28-B66F-8876A070F254}" name="Prueba 1"/>
     <tableColumn id="2" xr3:uid="{76608C69-5FD7-4DD4-97E2-6FBABBC30ABA}" name="Prueba 2"/>
     <tableColumn id="3" xr3:uid="{89FAED6E-C093-450B-9ED6-3D6298792216}" name="Prueba 3"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{0D7C2B78-B27D-4399-89FD-8EFF20562257}" name="Tabla13" displayName="Tabla13" ref="A7:C10" totalsRowShown="0">
+  <autoFilter ref="A7:C10" xr:uid="{0D7C2B78-B27D-4399-89FD-8EFF20562257}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{E236A14A-958D-4F09-B166-91450275DFEA}" name="Prueba 1"/>
+    <tableColumn id="2" xr3:uid="{A6D590E7-9757-4824-AEB4-EE3FE95EDCF1}" name="Prueba 2"/>
+    <tableColumn id="3" xr3:uid="{187BF580-057B-4C27-B4FB-5951B5412361}" name="Prueba 3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -378,61 +393,126 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="0" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="3" width="10.85546875" customWidth="1"/>
+    <col min="1" max="3" width="10.88671875" customWidth="1"/>
+    <col min="4" max="4" width="9.109375" customWidth="1"/>
+    <col min="5" max="16384" width="9.109375" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1">
+        <v>1880</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B3" t="s">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B4" t="s">
         <v>5</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>5</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B5" t="s">
         <v>3</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C5" t="s">
         <v>3</v>
       </c>
     </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>1884</v>
+      </c>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A6:C6"/>
+  </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
+  <tableParts count="2">
     <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>